<commit_message>
Auto: Weekly update of data
</commit_message>
<xml_diff>
--- a/datasets/xlsx/CSFaceit.xlsx
+++ b/datasets/xlsx/CSFaceit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\avery\OneDrive\Desktop\CS2 Project\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73D764BE-97B2-4619-98E3-52A656244EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA961C9B-3D06-4F9C-B7F9-510596D0B785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-24120" yWindow="7965" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31405,6 +31405,12 @@
         <f t="shared" si="33"/>
         <v>4.1666666666666664E-2</v>
       </c>
+      <c r="U329">
+        <v>1112</v>
+      </c>
+      <c r="V329">
+        <v>4</v>
+      </c>
       <c r="AA329">
         <f t="shared" si="29"/>
         <v>0</v>

</xml_diff>